<commit_message>
Changed beef exports to avoid problems due to organic --> conventional calf redist
</commit_message>
<xml_diff>
--- a/data/scenarios/food_as_culture.xlsx
+++ b/data/scenarios/food_as_culture.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1239" uniqueCount="211">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1240" uniqueCount="212">
   <si>
     <t>f_food</t>
   </si>
@@ -661,6 +661,9 @@
   </si>
   <si>
     <t>processing</t>
+  </si>
+  <si>
+    <t>JK: Changed to abs here as 0 in default</t>
   </si>
 </sst>
 </file>
@@ -9342,10 +9345,10 @@
         <v>179</v>
       </c>
       <c r="G271" s="9" t="s">
-        <v>11</v>
+        <v>96</v>
       </c>
       <c r="H271" s="9">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I271" s="9"/>
       <c r="J271" s="9"/>
@@ -9353,9 +9356,12 @@
       <c r="L271" s="9"/>
       <c r="M271" s="9"/>
       <c r="N271" s="9">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="O271" s="34"/>
+      <c r="P271" s="4" t="s">
+        <v>211</v>
+      </c>
       <c r="Q271" s="9"/>
       <c r="R271" s="9"/>
       <c r="S271" s="9"/>

</xml_diff>

<commit_message>
Fix in scenarios to avoid unfeasibility due to 'redist_*_calves' parameters
</commit_message>
<xml_diff>
--- a/data/scenarios/food_as_culture.xlsx
+++ b/data/scenarios/food_as_culture.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="164011"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="18360" windowHeight="6615" activeTab="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="18360" windowHeight="6615" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="Regions" sheetId="7" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1240" uniqueCount="212">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1241" uniqueCount="213">
   <si>
     <t>f_food</t>
   </si>
@@ -664,6 +664,9 @@
   </si>
   <si>
     <t>JK: Changed to abs here as 0 in default</t>
+  </si>
+  <si>
+    <t>&lt;-- Unfeasibility problems if this does not reach zero by 2040</t>
   </si>
 </sst>
 </file>
@@ -674,7 +677,7 @@
     <numFmt numFmtId="164" formatCode="0.0"/>
     <numFmt numFmtId="165" formatCode="0.0000"/>
   </numFmts>
-  <fonts count="12" x14ac:knownFonts="1">
+  <fonts count="13" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -761,6 +764,13 @@
       <sz val="11"/>
       <name val="Calibri"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="4"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="5">
@@ -883,7 +893,7 @@
     <xf numFmtId="9" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="55">
+  <cellXfs count="56">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -939,6 +949,7 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="165" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -10756,7 +10767,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:M13"/>
+  <dimension ref="A1:N13"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="8" bestFit="1" customWidth="1"/>
@@ -10768,7 +10779,7 @@
     <col min="7" max="13" width="7" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>97</v>
       </c>
@@ -10809,7 +10820,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>98</v>
       </c>
@@ -10834,7 +10845,7 @@
         <v>0.6</v>
       </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>98</v>
       </c>
@@ -10854,7 +10865,7 @@
         <v>0.6</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>98</v>
       </c>
@@ -10874,7 +10885,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>98</v>
       </c>
@@ -10894,7 +10905,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>123</v>
       </c>
@@ -10914,7 +10925,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>123</v>
       </c>
@@ -10934,7 +10945,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
       <c r="E9" t="s">
         <v>176</v>
       </c>
@@ -10944,11 +10955,17 @@
       <c r="G9" s="31">
         <v>1</v>
       </c>
+      <c r="K9">
+        <v>0</v>
+      </c>
       <c r="M9">
         <v>0</v>
       </c>
-    </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N9" s="55" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
       <c r="E10" t="s">
         <v>177</v>
       </c>
@@ -10958,11 +10975,14 @@
       <c r="G10" s="31">
         <v>1</v>
       </c>
+      <c r="K10">
+        <v>0</v>
+      </c>
       <c r="M10">
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>98</v>
       </c>
@@ -10982,7 +11002,7 @@
         <v>0.9</v>
       </c>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>123</v>
       </c>
@@ -11002,11 +11022,12 @@
         <v>0.9</v>
       </c>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:14" x14ac:dyDescent="0.25">
       <c r="G13" s="31"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>